<commit_message>
feat(productos): alta Antares Lager 660ml (cod 60022) + sumado a ACJ26-028
Codigo provisto por el usuario: 60022. Maestro 04D (CSV+xlsx) Cerveza Artesanal, lxu 0.66 (correcto para 660ml sin importar el pack). INOV_PRODUCTOS 19->20. Accion ACJ26-028 productos_marcas += 60022 (match por codigo). Validado: matchea 60022 y 60021, excluye lata 473. Cierra el pendiente del 660.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/04D_MAESTRO_PRODUCTOS_PENAFLOR.xlsx
+++ b/01_INPUTS/04D_MAESTRO_PRODUCTOS_PENAFLOR.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H259"/>
+  <dimension ref="A1:H260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -9676,6 +9676,42 @@
         <v>24</v>
       </c>
     </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Antares</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Cerveza Artesanal</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Cerveza Lager</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>60022</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Cerveza Artesanal</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>ANTARES LAGER 660 6X660 (60022)</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="H260" t="n">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>